<commit_message>
chores: update user story - Jingwei's proposal of dual signoff
</commit_message>
<xml_diff>
--- a/shared/CS-57_Contribution_Tracker.xlsx
+++ b/shared/CS-57_Contribution_Tracker.xlsx
@@ -12,7 +12,7 @@
   </sheets>
   <definedNames>
     <definedName hidden="1" localSheetId="1" name="_xlnm._FilterDatabase">'Contribution Log'!$A$1:$R$599</definedName>
-    <definedName hidden="1" localSheetId="3" name="_xlnm._FilterDatabase">'Jira Statistics'!$B$52:$K$144</definedName>
+    <definedName hidden="1" localSheetId="3" name="_xlnm._FilterDatabase">'Jira Statistics'!$B$52:$K$145</definedName>
   </definedNames>
   <calcPr fullCalcOnLoad="1"/>
 </workbook>
@@ -34133,11 +34133,11 @@
     </row>
     <row r="6" ht="30.0" customHeight="1">
       <c r="B6" s="27">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C6" s="14"/>
       <c r="D6" s="27">
-        <v>4.0</v>
+        <v>5</v>
       </c>
       <c r="E6" s="14"/>
       <c r="F6" s="27">
@@ -34145,11 +34145,11 @@
       </c>
       <c r="G6" s="14"/>
       <c r="H6" s="27">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="I6" s="14"/>
       <c r="J6" s="27">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="K6" s="14"/>
       <c r="L6" s="27">
@@ -34951,26 +34951,26 @@
         <v>Jingwei Lin</v>
       </c>
       <c r="C43" s="61">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D43" s="20">
         <v>0</v>
       </c>
       <c r="E43" s="20">
-        <v>0.0</v>
+        <v>1</v>
       </c>
       <c r="F43" s="20">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G43" s="20">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="H43" s="20">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I43" s="62" t="inlineStr">
         <is>
-          <t xml:space="preserve">Project setup &amp; status UI, Task &amp; item backend, Draft ownership &amp; verdict, Review, permissions &amp; dispute, Audit &amp; history, Unallocated, Release &amp; export, Annotation page &amp; judgement</t>
+          <t xml:space="preserve">Project setup &amp; status UI, Task &amp; item backend, Draft ownership &amp; verdict, Review, permissions &amp; dispute, Audit &amp; history, Unallocated, Annotation page &amp; judgement</t>
         </is>
       </c>
       <c r="J43" s="16">
@@ -35029,10 +35029,10 @@
         <v>0</v>
       </c>
       <c r="E45" s="20">
-        <v>1.0</v>
+        <v>0</v>
       </c>
       <c r="F45" s="20">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G45" s="20">
         <v>11</v>
@@ -35168,7 +35168,7 @@
       </c>
       <c r="D49" s="65" t="inlineStr">
         <is>
-          <t xml:space="preserve">11 of 92 issues on the board have no owner.</t>
+          <t xml:space="preserve">11 of 93 issues on the board have no owner.</t>
         </is>
       </c>
       <c r="E49" s="55"/>
@@ -36675,7 +36675,7 @@
       </c>
       <c r="D97" s="61" t="inlineStr">
         <is>
-          <t xml:space="preserve">In Review</t>
+          <t xml:space="preserve">Done</t>
         </is>
       </c>
       <c r="E97" s="20" t="s">
@@ -36730,7 +36730,7 @@
       </c>
       <c r="I98" s="61" t="inlineStr">
         <is>
-          <t xml:space="preserve">A1, H5, I4</t>
+          <t xml:space="preserve">I4</t>
         </is>
       </c>
       <c r="J98" s="66" t="s">
@@ -37698,7 +37698,7 @@
       </c>
       <c r="D127" s="61" t="inlineStr">
         <is>
-          <t xml:space="preserve">In Progress</t>
+          <t xml:space="preserve">In Review</t>
         </is>
       </c>
       <c r="E127" s="20" t="inlineStr">
@@ -38135,8 +38135,10 @@
       <c r="C140" s="20" t="s">
         <v>356</v>
       </c>
-      <c r="D140" s="61" t="s">
-        <v>447</v>
+      <c r="D140" s="61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">In Progress</t>
+        </is>
       </c>
       <c r="E140" s="20"/>
       <c r="F140" s="20" t="inlineStr">
@@ -38302,7 +38304,7 @@
       </c>
       <c r="I144" s="61" t="inlineStr">
         <is>
-          <t xml:space="preserve">A1, H5</t>
+          <t xml:space="preserve">A1, A4, H5</t>
         </is>
       </c>
       <c r="J144" s="66" t="inlineStr">
@@ -38314,7 +38316,56 @@
         <f>COUNTIF('Contribution Log'!$F$2:$F$596,$B144)</f>
       </c>
     </row>
-    <row r="145" ht="13.5" customHeight="1"/>
+    <row r="145" ht="13.5" customHeight="1">
+      <c r="B145" s="61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SCRUM-126</t>
+        </is>
+      </c>
+      <c r="C145" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Task</t>
+        </is>
+      </c>
+      <c r="D145" s="61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">In Progress</t>
+        </is>
+      </c>
+      <c r="E145" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jingwei Lin</t>
+        </is>
+      </c>
+      <c r="F145" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">W10 Gate releases, prove them</t>
+        </is>
+      </c>
+      <c r="G145" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Review, Dispute &amp; Adjudication</t>
+        </is>
+      </c>
+      <c r="H145" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dispute: An independent reviewer can settle a held disagreement, except where adjudication is mandatory</t>
+        </is>
+      </c>
+      <c r="I145" s="61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">E5, G2</t>
+        </is>
+      </c>
+      <c r="J145" s="66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">description</t>
+        </is>
+      </c>
+      <c r="K145" s="16">
+        <f>COUNTIF('Contribution Log'!$F$2:$F$596,$B145)</f>
+      </c>
+    </row>
     <row r="146" ht="13.5" customHeight="1"/>
     <row r="147" ht="13.5" customHeight="1"/>
     <row r="148" ht="13.5" customHeight="1"/>
@@ -39171,7 +39222,7 @@
     <row r="999" ht="15.75" customHeight="1"/>
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
-  <autoFilter ref="$B$52:$K$144"/>
+  <autoFilter ref="$B$52:$K$145"/>
   <mergeCells count="26">
     <mergeCell ref="H6:I6"/>
     <mergeCell ref="J6:K6"/>
@@ -39200,17 +39251,17 @@
     <mergeCell ref="D19:E19"/>
     <mergeCell ref="C36:K36"/>
   </mergeCells>
-  <conditionalFormatting sqref="B53:K144">
+  <conditionalFormatting sqref="B53:K145">
     <cfRule type="expression" dxfId="1" priority="1">
       <formula>$D53="Done"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B53:K144">
+  <conditionalFormatting sqref="B53:K145">
     <cfRule type="expression" dxfId="0" priority="2">
       <formula>$D53="In Progress"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B53:K144">
+  <conditionalFormatting sqref="B53:K145">
     <cfRule type="expression" dxfId="2" priority="3">
       <formula>$D53="In Review"</formula>
     </cfRule>
@@ -39220,7 +39271,7 @@
       <formula>3</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I53:I144">
+  <conditionalFormatting sqref="I53:I145">
     <cfRule type="expression" dxfId="3" priority="5">
       <formula>$I53=""</formula>
     </cfRule>
@@ -40792,7 +40843,7 @@
       </c>
       <c r="P3" s="59" t="inlineStr">
         <is>
-          <t xml:space="preserve">SCRUM-73, SCRUM-125</t>
+          <t xml:space="preserve">SCRUM-125</t>
         </is>
       </c>
       <c r="T3" s="69" t="s">
@@ -40962,8 +41013,10 @@
       <c r="O6" s="59" t="s">
         <v>453</v>
       </c>
-      <c r="P6" s="59" t="s">
-        <v>454</v>
+      <c r="P6" s="59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SCRUM-84, SCRUM-125</t>
+        </is>
       </c>
       <c r="T6" s="69" t="s">
         <v>336</v>
@@ -40979,8 +41032,10 @@
       <c r="X6" s="59" t="s">
         <v>221</v>
       </c>
-      <c r="Y6" s="59" t="s">
-        <v>129</v>
+      <c r="Y6" s="59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">In progress</t>
+        </is>
       </c>
       <c r="Z6" s="59" t="s">
         <v>153</v>
@@ -41833,15 +41888,17 @@
       <c r="O31" s="59" t="s">
         <v>537</v>
       </c>
-      <c r="P31" s="59" t="s">
-        <v>538</v>
+      <c r="P31" s="59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SCRUM-107, SCRUM-126</t>
+        </is>
       </c>
       <c r="X31" s="59" t="s">
         <v>191</v>
       </c>
       <c r="Y31" s="59" t="inlineStr">
         <is>
-          <t xml:space="preserve">Done</t>
+          <t xml:space="preserve">In progress</t>
         </is>
       </c>
       <c r="Z31" s="59" t="s">
@@ -42075,15 +42132,17 @@
       <c r="O39" s="59" t="s">
         <v>561</v>
       </c>
-      <c r="P39" s="59" t="s">
-        <v>562</v>
+      <c r="P39" s="59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SCRUM-50, SCRUM-107, SCRUM-118, SCRUM-126</t>
+        </is>
       </c>
       <c r="X39" s="59" t="s">
         <v>221</v>
       </c>
       <c r="Y39" s="59" t="inlineStr">
         <is>
-          <t xml:space="preserve">Done</t>
+          <t xml:space="preserve">In progress</t>
         </is>
       </c>
       <c r="Z39" s="59" t="s">
@@ -42319,7 +42378,7 @@
       </c>
       <c r="P47" s="59" t="inlineStr">
         <is>
-          <t xml:space="preserve">SCRUM-43, SCRUM-73, SCRUM-125</t>
+          <t xml:space="preserve">SCRUM-43, SCRUM-125</t>
         </is>
       </c>
       <c r="X47" s="59" t="s">
@@ -42449,7 +42508,7 @@
       </c>
       <c r="Y51" s="59" t="inlineStr">
         <is>
-          <t xml:space="preserve">In progress</t>
+          <t xml:space="preserve">Done</t>
         </is>
       </c>
       <c r="Z51" s="59" t="s">
@@ -43006,7 +43065,13 @@
         </is>
       </c>
     </row>
-    <row r="94" ht="13.5" customHeight="1"/>
+    <row r="94" ht="13.5" customHeight="1">
+      <c r="Z94" s="59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SCRUM-126</t>
+        </is>
+      </c>
+    </row>
     <row r="95" ht="13.5" customHeight="1"/>
     <row r="96" ht="13.5" customHeight="1"/>
     <row r="97" ht="13.5" customHeight="1"/>

</xml_diff>